<commit_message>
Major performance improvements when dealing with conditional formats. Minor performance improvements across the board.
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/AutoFilter/CustomAutoFilter.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/AutoFilter/CustomAutoFilter.xlsx
@@ -58,7 +58,21 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="3">
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>

</xml_diff>